<commit_message>
Committing BR comments on escalation tracker
</commit_message>
<xml_diff>
--- a/escalation_tracker.xlsx
+++ b/escalation_tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brendan/GitHub/projects/moalmanac-db-hscni/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E6CF009-5587-7043-952D-C2FDC55D03C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DA5F829-470B-394A-8073-599B011CF675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19140" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8040" yWindow="740" windowWidth="28660" windowHeight="17120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="912" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="943" uniqueCount="340">
   <si>
     <t>NI-MOAlmanac — Brendan Escalation Tracker</t>
   </si>
@@ -953,6 +953,99 @@
   </si>
   <si>
     <t>0, 1, 2, 3, 4, 5, 6, 7, 8, 792, 793, 794</t>
+  </si>
+  <si>
+    <t>BCR::ABL1 is the correct proxy</t>
+  </si>
+  <si>
+    <t>Yes, these woul be BRCA1/2 pathogenic variants</t>
+  </si>
+  <si>
+    <t>Yes this is correct</t>
+  </si>
+  <si>
+    <t>28, 840</t>
+  </si>
+  <si>
+    <t>This depends on the specific approval and underlying clinical trials. What specific indications are this row referencing?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes, HR+ is split between ER+ / PR-, ER-/PR+, and ER+/PR+. This is because the GA4GH schema does not yet support multiple biomarkers being combined in series or with "OR" logic. </t>
+  </si>
+  <si>
+    <t>Correct. Triple negative is HER2-, ER-, and PR-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes, there are separate relationships for NTRK1, NTRK2, and NTRK3. </t>
+  </si>
+  <si>
+    <t>Larotrectinib: 199, 200, 201; Entrectinib: 121, 122, 123; Repotrectinib: 369, 370, 371</t>
+  </si>
+  <si>
+    <t>Yes, we don't consider stage w.r.t. cancer type. ind:nice.ta569:1.1 includes "in combination with chemotherapy", so we should find out what chemotherapies were offered in the supporting trial to determine which proposition(s) to associate. TA362 would be proposition 20</t>
+  </si>
+  <si>
+    <t>20 for TA632</t>
+  </si>
+  <si>
+    <t>We've been coding things as "ALL". The most updated versions of OncoTree dropped "BALL" and "ALL". We are soon~ish going to switch to the NCI Thesaurus as a primary coding with mappings to oncotree. So, I'd stick with Acute Lymphoid Leukemia as a Coding. (disease id == 0)</t>
+  </si>
+  <si>
+    <t>According to the NICE document for this indication, this is based on KEYNOTE-859, and thus the analog approval is this one from the FDA: https://ie.moalmanac.org/indications/ind:fda.keytruda:7. We thus need to make two new propositions that include the CPS &gt;=1 criteria. I can do that once a JSON is created for the indication because we'll also want to update the statement text like we did with the FDA indication. I wonder if it is worthwhile adding some of the commentary from the NICE approval into the statement text, such as a summary of the overall decision to include the CPS criteria (section 3.16 of the NICE approval: https://www.nice.org.uk/guidance/ta997/resources/pembrolizumab-with-platinum-and-fluoropyrimidinebased-chemotherapy-for-untreated-advanced-her2negative-gastric-or-gastrooesophageal-junction-adenocarcinoma-pdf-82615975905733)</t>
+  </si>
+  <si>
+    <t>Per row 48, we'll have to create new propositions for the two chemotherapy agents used in combination with pembrolizumab based on KEYNOTE-859</t>
+  </si>
+  <si>
+    <t>Thanks for catching this re: midostaurin + cytarabine! For quizartinib + cytarabine, I think that this would be the same proposition, right? https://ie.moalmanac.org/indications/ind:hse.00886:a. Hm… based on the underlying clinical trial, it looks like they also offered idarubicin (https://pubmed.ncbi.nlm.nih.gov/37116523/) as the anthracycline. We can create a new proposition for this</t>
+  </si>
+  <si>
+    <t>The approval specifically lists CD22 positive status as eligibility criteria, so this is an included biomarker. The EMA also includes the BCR::ABL1 comment (https://ie.moalmanac.org/indications/ind:ema.besponsa:0), so we derived two propositions for the EMA equivalent.</t>
+  </si>
+  <si>
+    <t>168, 543</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TA589 and TA1049 both list CD19-positive status as an eligibility criteria, so CD19+ is a biomarker. NICE also includes BCR::ABL1 negative status as a requirement whereas the FDA does not (https://ie.moalmanac.org/indications/ind:fda.blincyto:0) so I think that we'll need to create a new proposition. </t>
+  </si>
+  <si>
+    <t>biomarker 15 is BCR::ABL1 negative, so relevant propositions will include that biomarker. This isn't displayed well on the site and needs to be updated. TA450: will need new propositions because NICE dropped the CD- status requirement; TA589: ; TA1049:... Brendan will return to this once refactoring biomarker negative statuses</t>
+  </si>
+  <si>
+    <t>Can you expand upon this one? I'm not quite understanding the Issue Summary.</t>
+  </si>
+  <si>
+    <t>Correct. MOAlmanac doesn't consider phase or stage of cancer types.</t>
+  </si>
+  <si>
+    <t>Brendan will return to this after refactoring negative relationships.</t>
+  </si>
+  <si>
+    <t>We haven't included MRD criteria in any relationships per not considering stage or phase of cancer type</t>
+  </si>
+  <si>
+    <t>Whoops! Thank you for catching this! Adding an Issue to update these entries.</t>
+  </si>
+  <si>
+    <t>Thanks for catching this! You should still map to the appropriate proposition, the therapy strategy won't impact the proposition</t>
+  </si>
+  <si>
+    <t>Thanks for catching this!</t>
+  </si>
+  <si>
+    <t>MRD is not considered a biomarker and moalmanac doesn't consider stage/phase within the cancer type</t>
+  </si>
+  <si>
+    <t>Not applicable, I think? No current db entries are based on NICE approvals</t>
+  </si>
+  <si>
+    <t>This ends up being derived as esophagogastric adenocarcinoma, gastrointestinal stromal tumor, and cholangiocarcinoma. You can follow this approval: http://localhost:4000/indications/ind:ema.keytruda:8. Rather than splitting nice.ta914b into three indications, i'd leave it as one because the indication text is supposed to be "as written" by the approval agency.</t>
+  </si>
+  <si>
+    <t>Treatment history can be included as part of the indication or statement text, depending on how it is written. We don't consider treatment history within eligibility criteria for moalmanac propositions though. I'd include this in the indication text based on reading TA1021 in your indications spreadsheet.</t>
+  </si>
+  <si>
+    <t>MOAlmanac doesn't consider line of therapy or switch maintenance, those clinical details should be noted. However, we should create a new proposition since this indication is for "EGFR TK variants", not EGFR activating variants. I'll have to look at the NICE text and the FDA approval more closely. EMA has broadly approved this indication for "EGFR activating variants" and the FDA explicitly did for p.L858R and exon 19 deletions.</t>
   </si>
 </sst>
 </file>
@@ -1116,7 +1209,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1183,13 +1276,6 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1201,6 +1287,19 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="43" fontId="7" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1516,20 +1615,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="2" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -1662,10 +1761,10 @@
       <c r="H1" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="31" t="s">
+      <c r="I1" s="28" t="s">
         <v>301</v>
       </c>
-      <c r="J1" s="31" t="s">
+      <c r="J1" s="28" t="s">
         <v>302</v>
       </c>
     </row>
@@ -2059,7 +2158,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="19">
         <v>16</v>
       </c>
@@ -2085,7 +2184,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="15">
         <v>17</v>
       </c>
@@ -2111,7 +2210,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="19">
         <v>18</v>
       </c>
@@ -2137,7 +2236,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="15">
         <v>19</v>
       </c>
@@ -2163,7 +2262,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="19">
         <v>20</v>
       </c>
@@ -2189,7 +2288,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="15">
         <v>21</v>
       </c>
@@ -2215,7 +2314,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="19">
         <v>22</v>
       </c>
@@ -2241,7 +2340,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="15">
         <v>23</v>
       </c>
@@ -2267,7 +2366,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="19">
         <v>24</v>
       </c>
@@ -2293,7 +2392,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="15">
         <v>25</v>
       </c>
@@ -2319,7 +2418,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="19">
         <v>26</v>
       </c>
@@ -2345,7 +2444,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="15">
         <v>27</v>
       </c>
@@ -2371,7 +2470,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="19">
         <v>28</v>
       </c>
@@ -2397,7 +2496,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="15">
         <v>29</v>
       </c>
@@ -2423,7 +2522,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="19">
         <v>30</v>
       </c>
@@ -2448,8 +2547,11 @@
       <c r="H31" s="21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I31" s="36" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="15">
         <v>31</v>
       </c>
@@ -2474,8 +2576,11 @@
       <c r="H32" s="18" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I32" s="37" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="19">
         <v>32</v>
       </c>
@@ -2500,8 +2605,11 @@
       <c r="H33" s="21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I33" s="36" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="15">
         <v>33</v>
       </c>
@@ -2526,8 +2634,11 @@
       <c r="H34" s="18" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I34" s="37" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="19">
         <v>34</v>
       </c>
@@ -2552,8 +2663,11 @@
       <c r="H35" s="21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I35" s="36" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="15">
         <v>35</v>
       </c>
@@ -2578,8 +2692,11 @@
       <c r="H36" s="18" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I36" s="37" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="19">
         <v>36</v>
       </c>
@@ -2604,8 +2721,11 @@
       <c r="H37" s="21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I37" s="36" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="15">
         <v>37</v>
       </c>
@@ -2630,8 +2750,11 @@
       <c r="H38" s="18" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I38" s="37" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="19">
         <v>38</v>
       </c>
@@ -2656,8 +2779,11 @@
       <c r="H39" s="21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I39" s="36" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="15">
         <v>39</v>
       </c>
@@ -2682,8 +2808,11 @@
       <c r="H40" s="18" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I40" s="37" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="19">
         <v>40</v>
       </c>
@@ -2708,8 +2837,11 @@
       <c r="H41" s="21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I41" s="36" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="15">
         <v>41</v>
       </c>
@@ -2734,8 +2866,11 @@
       <c r="H42" s="18" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I42" s="37" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="19">
         <v>42</v>
       </c>
@@ -2760,8 +2895,11 @@
       <c r="H43" s="21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I43" s="36" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="15">
         <v>43</v>
       </c>
@@ -2786,8 +2924,11 @@
       <c r="H44" s="18" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I44" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="19">
         <v>44</v>
       </c>
@@ -2812,8 +2953,14 @@
       <c r="H45" s="21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I45" s="36" t="s">
+        <v>324</v>
+      </c>
+      <c r="J45" s="36" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="15">
         <v>45</v>
       </c>
@@ -2838,8 +2985,11 @@
       <c r="H46" s="18" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="47" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I46" s="30" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="19">
         <v>46</v>
       </c>
@@ -2864,8 +3014,11 @@
       <c r="H47" s="21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I47" s="31" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="15">
         <v>47</v>
       </c>
@@ -2889,6 +3042,9 @@
       </c>
       <c r="H48" s="18" t="s">
         <v>28</v>
+      </c>
+      <c r="I48" s="30" t="s">
+        <v>321</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -2916,6 +3072,9 @@
       <c r="H49" s="21" t="s">
         <v>28</v>
       </c>
+      <c r="I49" s="31" t="s">
+        <v>320</v>
+      </c>
     </row>
     <row r="50" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="15">
@@ -2942,6 +3101,9 @@
       <c r="H50" s="18" t="s">
         <v>28</v>
       </c>
+      <c r="I50" s="30" t="s">
+        <v>309</v>
+      </c>
     </row>
     <row r="51" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="19">
@@ -2968,6 +3130,12 @@
       <c r="H51" s="21" t="s">
         <v>28</v>
       </c>
+      <c r="I51" s="31" t="s">
+        <v>311</v>
+      </c>
+      <c r="J51" s="31" t="s">
+        <v>312</v>
+      </c>
     </row>
     <row r="52" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="15">
@@ -2994,6 +3162,12 @@
       <c r="H52" s="18" t="s">
         <v>28</v>
       </c>
+      <c r="I52" s="30" t="s">
+        <v>318</v>
+      </c>
+      <c r="J52" s="30" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="53" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="19">
@@ -3020,6 +3194,12 @@
       <c r="H53" s="21" t="s">
         <v>28</v>
       </c>
+      <c r="I53" s="31" t="s">
+        <v>316</v>
+      </c>
+      <c r="J53" s="31" t="s">
+        <v>317</v>
+      </c>
     </row>
     <row r="54" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="15">
@@ -3046,6 +3226,9 @@
       <c r="H54" s="18" t="s">
         <v>28</v>
       </c>
+      <c r="I54" s="30" t="s">
+        <v>315</v>
+      </c>
     </row>
     <row r="55" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="19">
@@ -3072,6 +3255,9 @@
       <c r="H55" s="21" t="s">
         <v>28</v>
       </c>
+      <c r="I55" s="31" t="s">
+        <v>314</v>
+      </c>
     </row>
     <row r="56" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="15">
@@ -3098,6 +3284,9 @@
       <c r="H56" s="18" t="s">
         <v>28</v>
       </c>
+      <c r="I56" s="30" t="s">
+        <v>310</v>
+      </c>
     </row>
     <row r="57" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="19">
@@ -3124,6 +3313,9 @@
       <c r="H57" s="21" t="s">
         <v>28</v>
       </c>
+      <c r="I57" s="31" t="s">
+        <v>313</v>
+      </c>
     </row>
     <row r="58" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="15">
@@ -3150,7 +3342,7 @@
       <c r="H58" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="I58" s="35" t="s">
+      <c r="I58" s="32" t="s">
         <v>307</v>
       </c>
       <c r="J58" t="s">
@@ -3182,7 +3374,7 @@
       <c r="H59" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I59" s="34" t="s">
+      <c r="I59" s="31" t="s">
         <v>306</v>
       </c>
     </row>
@@ -3211,10 +3403,10 @@
       <c r="H60" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="I60" s="33" t="s">
+      <c r="I60" s="30" t="s">
         <v>304</v>
       </c>
-      <c r="J60" s="33" t="s">
+      <c r="J60" s="30" t="s">
         <v>305</v>
       </c>
     </row>
@@ -3243,7 +3435,7 @@
       <c r="H61" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I61" s="32" t="s">
+      <c r="I61" s="29" t="s">
         <v>303</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Brendan comments, 6 left
</commit_message>
<xml_diff>
--- a/escalation_tracker.xlsx
+++ b/escalation_tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brendan/GitHub/projects/moalmanac-db-hscni/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DA5F829-470B-394A-8073-599B011CF675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{229AB91F-9DD6-A840-9630-183FCD1E5384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8040" yWindow="740" windowWidth="28660" windowHeight="17120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3540" yWindow="700" windowWidth="31400" windowHeight="25580" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="943" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="975" uniqueCount="368">
   <si>
     <t>NI-MOAlmanac — Brendan Escalation Tracker</t>
   </si>
@@ -1046,6 +1046,91 @@
   </si>
   <si>
     <t>MOAlmanac doesn't consider line of therapy or switch maintenance, those clinical details should be noted. However, we should create a new proposition since this indication is for "EGFR TK variants", not EGFR activating variants. I'll have to look at the NICE text and the FDA approval more closely. EMA has broadly approved this indication for "EGFR activating variants" and the FDA explicitly did for p.L858R and exon 19 deletions.</t>
+  </si>
+  <si>
+    <t>This does not involve a biomarker so we are not going to add it to moalmanac-db</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28, 840 </t>
+  </si>
+  <si>
+    <t>Propositions were present, see BR proposition(s) column</t>
+  </si>
+  <si>
+    <t>This derives to 15 relationships, see https://ie.moalmanac.org/indications/ind:fda.lynparza:1 for all of the propositions</t>
+  </si>
+  <si>
+    <t>243, 244, 245. 246, 247, 248, 249, 250, 251, 252, 253, 254, 255, 256, 257</t>
+  </si>
+  <si>
+    <t>Will need to create a new proposition</t>
+  </si>
+  <si>
+    <t>Will need to create new propositions for BRCA negative</t>
+  </si>
+  <si>
+    <t>223, 224, 225, 226, 227, 228</t>
+  </si>
+  <si>
+    <t>Will need to create new propositions for BRCA negative. Added propositions to the BR propositon(s) column for BRCA positive propositions.</t>
+  </si>
+  <si>
+    <t>Will need to create new propositions</t>
+  </si>
+  <si>
+    <t>This is an odd one. I am inclined to curate it as PD-L1 (TPS) &gt;= 0%. What do you think? They write this section in "Why the committee made these recommendations" Pembrolizumab combination therapy meets NICE's criteria to be considered a life-
+extending treatment at the end of life in both PD-L1 tumour proportion score subgroups. The cost-effectiveness estimates in people whose tumours express PD-L1 with a tumour proportion score of 0% to 49% were within what NICE considers a good use of NHS resources. For people whose tumours have a PD-L1 tumour proportion score of 50% or more and who need an urgent clinical intervention (for example, because their cancer may cause major airway blockage), the cost-effectiveness estimates were not certain. However, they are likely to be within what NICE considers a good use of NHS resources, so pembrolizumab combination is recommended in both groups."</t>
+  </si>
+  <si>
+    <t>This is the equivalent of this relationship: https://ie.moalmanac.org/indications/ind:ema.imfinzi:3</t>
+  </si>
+  <si>
+    <t>474, 475, 476, 477</t>
+  </si>
+  <si>
+    <t>We based this on the criteria used for eligibility in the underlying clinical trial: https://ie.moalmanac.org/indications/ind:ema.balversa:0 and also what the FDA companion diagnostics can assay for: https://www.fda.gov/medical-devices/in-vitro-diagnostics/list-cleared-or-approved-companion-diagnostic-devices-in-vitro-and-imaging-tools. I'll update the FDA, EMA, and HSE comments to specify that we used the companion diagnostic variants and remove fgfr3::baiap2l1.</t>
+  </si>
+  <si>
+    <t>At the moment we have these as separate propositions: https://ie.moalmanac.org/indications/ind:ema.tibsovo:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">190, 191, 192, 193, 194 </t>
+  </si>
+  <si>
+    <t>This is the equivalent of https://ie.moalmanac.org/indications/ind:ema.tecentriq:0</t>
+  </si>
+  <si>
+    <t>We only curated this as Bladder Urothelial Carcinoma because that makes up ~95% of cases, I am open to adding more though!</t>
+  </si>
+  <si>
+    <t>This is the equivalent of this: https://ie.moalmanac.org/indications/ind:ema.keytruda:12</t>
+  </si>
+  <si>
+    <t>335, 337</t>
+  </si>
+  <si>
+    <t>This is the equivalent of: https://ie.moalmanac.org/indications/ind:ema.ibrance:0</t>
+  </si>
+  <si>
+    <t>311, 312, 313</t>
+  </si>
+  <si>
+    <t>This is the equivalent of https://ie.moalmanac.org/indications/ind:ema.tecentriq:2 but the EMA does not require PD-L1 status. Will create a new proposition for PD-L1 &gt;= 0%</t>
+  </si>
+  <si>
+    <t>This is the equivalent of this relationship from the EMA: https://ie.moalmanac.org/indications/ind:ema.keytruda:11. Will need to create new propositions for PD-L1 (CPS) &gt;= 10 + PD-L1 (IC) &lt;= 1%</t>
+  </si>
+  <si>
+    <t>653, 654, 655</t>
+  </si>
+  <si>
+    <t>This is the equivalent of https://ie.moalmanac.org/indications/ind:ema.piqray:0. We didn't specify further beyond PIK3CA variants because the underlying clinical trial's enrollment criteria was broad. Removed TA1063 from this row since that is covered in the next one.</t>
+  </si>
+  <si>
+    <t>TA816</t>
+  </si>
+  <si>
+    <t>This is the equivalent of https://ie.moalmanac.org/indications/ind:ema.imfinzi:3</t>
   </si>
 </sst>
 </file>
@@ -1209,7 +1294,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1289,6 +1374,12 @@
     <xf numFmtId="43" fontId="7" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1296,11 +1387,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1615,20 +1703,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
     </row>
     <row r="2" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -1793,6 +1881,9 @@
       <c r="H2" s="18" t="s">
         <v>28</v>
       </c>
+      <c r="I2" s="34" t="s">
+        <v>349</v>
+      </c>
     </row>
     <row r="3" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="19">
@@ -1819,6 +1910,9 @@
       <c r="H3" s="21" t="s">
         <v>28</v>
       </c>
+      <c r="I3" s="38" t="s">
+        <v>350</v>
+      </c>
     </row>
     <row r="4" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="15">
@@ -1845,6 +1939,9 @@
       <c r="H4" s="18" t="s">
         <v>28</v>
       </c>
+      <c r="I4" s="34" t="s">
+        <v>349</v>
+      </c>
     </row>
     <row r="5" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="19">
@@ -1871,6 +1968,9 @@
       <c r="H5" s="21" t="s">
         <v>28</v>
       </c>
+      <c r="I5" s="33" t="s">
+        <v>345</v>
+      </c>
     </row>
     <row r="6" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="15">
@@ -1897,6 +1997,9 @@
       <c r="H6" s="18" t="s">
         <v>28</v>
       </c>
+      <c r="I6" s="34" t="s">
+        <v>346</v>
+      </c>
     </row>
     <row r="7" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="19">
@@ -1923,6 +2026,12 @@
       <c r="H7" s="21" t="s">
         <v>28</v>
       </c>
+      <c r="I7" s="33" t="s">
+        <v>348</v>
+      </c>
+      <c r="J7" s="33" t="s">
+        <v>347</v>
+      </c>
     </row>
     <row r="8" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15">
@@ -1948,6 +2057,12 @@
       </c>
       <c r="H8" s="18" t="s">
         <v>28</v>
+      </c>
+      <c r="I8" s="34" t="s">
+        <v>343</v>
+      </c>
+      <c r="J8" s="34" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -1975,6 +2090,9 @@
       <c r="H9" s="21" t="s">
         <v>28</v>
       </c>
+      <c r="I9" s="33" t="s">
+        <v>340</v>
+      </c>
     </row>
     <row r="10" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="15">
@@ -2001,6 +2119,12 @@
       <c r="H10" s="18" t="s">
         <v>28</v>
       </c>
+      <c r="I10" s="34" t="s">
+        <v>351</v>
+      </c>
+      <c r="J10" s="34" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="11" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="19">
@@ -2027,6 +2151,12 @@
       <c r="H11" s="21" t="s">
         <v>28</v>
       </c>
+      <c r="I11" s="33" t="s">
+        <v>342</v>
+      </c>
+      <c r="J11" t="s">
+        <v>341</v>
+      </c>
     </row>
     <row r="12" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="15">
@@ -2053,6 +2183,9 @@
       <c r="H12" s="18" t="s">
         <v>28</v>
       </c>
+      <c r="I12" s="33" t="s">
+        <v>340</v>
+      </c>
     </row>
     <row r="13" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="19">
@@ -2079,6 +2212,12 @@
       <c r="H13" s="21" t="s">
         <v>28</v>
       </c>
+      <c r="I13" s="33" t="s">
+        <v>342</v>
+      </c>
+      <c r="J13">
+        <v>877</v>
+      </c>
     </row>
     <row r="14" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="15">
@@ -2158,7 +2297,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="19">
         <v>16</v>
       </c>
@@ -2184,7 +2323,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="15">
         <v>17</v>
       </c>
@@ -2209,8 +2348,14 @@
       <c r="H18" s="18" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I18" s="34" t="s">
+        <v>367</v>
+      </c>
+      <c r="J18" s="34" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="19">
         <v>18</v>
       </c>
@@ -2236,7 +2381,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="15">
         <v>19</v>
       </c>
@@ -2262,12 +2407,12 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="19">
         <v>20</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>117</v>
+        <v>366</v>
       </c>
       <c r="C21" s="20" t="s">
         <v>118</v>
@@ -2287,8 +2432,14 @@
       <c r="H21" s="21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I21" s="33" t="s">
+        <v>365</v>
+      </c>
+      <c r="J21" s="33" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="15">
         <v>21</v>
       </c>
@@ -2313,8 +2464,11 @@
       <c r="H22" s="18" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I22" s="34" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="19">
         <v>22</v>
       </c>
@@ -2339,8 +2493,11 @@
       <c r="H23" s="21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I23" s="33" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="15">
         <v>23</v>
       </c>
@@ -2365,8 +2522,11 @@
       <c r="H24" s="18" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I24" s="34" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="19">
         <v>24</v>
       </c>
@@ -2391,8 +2551,14 @@
       <c r="H25" s="21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I25" s="33" t="s">
+        <v>360</v>
+      </c>
+      <c r="J25" s="33" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="15">
         <v>25</v>
       </c>
@@ -2417,8 +2583,14 @@
       <c r="H26" s="18" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I26" s="34" t="s">
+        <v>358</v>
+      </c>
+      <c r="J26" s="34" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="19">
         <v>26</v>
       </c>
@@ -2443,8 +2615,14 @@
       <c r="H27" s="21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I27" s="33" t="s">
+        <v>357</v>
+      </c>
+      <c r="J27">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="15">
         <v>27</v>
       </c>
@@ -2469,8 +2647,14 @@
       <c r="H28" s="18" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="29" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I28" s="34" t="s">
+        <v>356</v>
+      </c>
+      <c r="J28">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="19">
         <v>28</v>
       </c>
@@ -2495,8 +2679,14 @@
       <c r="H29" s="21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I29" s="33" t="s">
+        <v>354</v>
+      </c>
+      <c r="J29" s="33" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="15">
         <v>29</v>
       </c>
@@ -2521,8 +2711,11 @@
       <c r="H30" s="18" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I30" s="34" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="19">
         <v>30</v>
       </c>
@@ -2547,11 +2740,11 @@
       <c r="H31" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I31" s="36" t="s">
+      <c r="I31" s="33" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="15">
         <v>31</v>
       </c>
@@ -2576,7 +2769,7 @@
       <c r="H32" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="I32" s="37" t="s">
+      <c r="I32" s="34" t="s">
         <v>338</v>
       </c>
     </row>
@@ -2605,7 +2798,7 @@
       <c r="H33" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I33" s="36" t="s">
+      <c r="I33" s="33" t="s">
         <v>337</v>
       </c>
     </row>
@@ -2634,7 +2827,7 @@
       <c r="H34" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="I34" s="37" t="s">
+      <c r="I34" s="34" t="s">
         <v>336</v>
       </c>
     </row>
@@ -2663,7 +2856,7 @@
       <c r="H35" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I35" s="36" t="s">
+      <c r="I35" s="33" t="s">
         <v>335</v>
       </c>
     </row>
@@ -2692,7 +2885,7 @@
       <c r="H36" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="I36" s="37" t="s">
+      <c r="I36" s="34" t="s">
         <v>334</v>
       </c>
     </row>
@@ -2721,7 +2914,7 @@
       <c r="H37" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I37" s="36" t="s">
+      <c r="I37" s="33" t="s">
         <v>333</v>
       </c>
     </row>
@@ -2750,7 +2943,7 @@
       <c r="H38" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="I38" s="37" t="s">
+      <c r="I38" s="34" t="s">
         <v>332</v>
       </c>
     </row>
@@ -2779,7 +2972,7 @@
       <c r="H39" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I39" s="36" t="s">
+      <c r="I39" s="33" t="s">
         <v>331</v>
       </c>
     </row>
@@ -2808,7 +3001,7 @@
       <c r="H40" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="I40" s="37" t="s">
+      <c r="I40" s="34" t="s">
         <v>330</v>
       </c>
     </row>
@@ -2837,7 +3030,7 @@
       <c r="H41" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I41" s="36" t="s">
+      <c r="I41" s="33" t="s">
         <v>329</v>
       </c>
     </row>
@@ -2866,7 +3059,7 @@
       <c r="H42" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="I42" s="37" t="s">
+      <c r="I42" s="34" t="s">
         <v>328</v>
       </c>
     </row>
@@ -2895,7 +3088,7 @@
       <c r="H43" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I43" s="36" t="s">
+      <c r="I43" s="33" t="s">
         <v>327</v>
       </c>
     </row>
@@ -2953,10 +3146,10 @@
       <c r="H45" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I45" s="36" t="s">
+      <c r="I45" s="33" t="s">
         <v>324</v>
       </c>
-      <c r="J45" s="36" t="s">
+      <c r="J45" s="33" t="s">
         <v>325</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Finished review of addressable escalations w/o needing new propositions
</commit_message>
<xml_diff>
--- a/escalation_tracker.xlsx
+++ b/escalation_tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brendan/GitHub/projects/moalmanac-db-hscni/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{229AB91F-9DD6-A840-9630-183FCD1E5384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{380BB488-14FF-8C4C-864A-B5AF958CE543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3540" yWindow="700" windowWidth="31400" windowHeight="25580" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="220" yWindow="600" windowWidth="31400" windowHeight="19140" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="975" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1023" uniqueCount="413">
   <si>
     <t>NI-MOAlmanac — Brendan Escalation Tracker</t>
   </si>
@@ -1131,6 +1131,141 @@
   </si>
   <si>
     <t>This is the equivalent of https://ie.moalmanac.org/indications/ind:ema.imfinzi:3</t>
+  </si>
+  <si>
+    <t>TA1086</t>
+  </si>
+  <si>
+    <t>TA632</t>
+  </si>
+  <si>
+    <t>TA569</t>
+  </si>
+  <si>
+    <t>ribociclib with aromatase inhibitor</t>
+  </si>
+  <si>
+    <t>HR+, HER2- breast cancer</t>
+  </si>
+  <si>
+    <t>This is equivalent to this approval: https://dev.moalmanac.org/indications/ind:ema.kisqali:1. Add "This indication is based on NATALEE (NCT03701334) was a randomized (1:1), open-label, multicenter study, where participants received goserelin and either letrozole or anastrozole, in addition to ribociclib." to the indication's description.</t>
+  </si>
+  <si>
+    <t>499, 500, 501, 502, 503, 504</t>
+  </si>
+  <si>
+    <t>Abemaciclib with endocrine therapy</t>
+  </si>
+  <si>
+    <t>This is the equivlant of this approval: https://dev.moalmanac.org/indications/ind:ema.verzenios:0. Add "The product information further states that this indication was approved based on results from the monarchE study, a randomized, open label, two cohort, phase 3 study which enrolled a total of 5,637 patients who were randomized in a 1:1 ratio to receive 2 years of abemaciclib plus physician's choice of standard endocrine therapy, or standard endocrine therapy alone. Initial endocrine therapy received by patients included letrozole (39%), tamoxifen (31%), anastrozole (22%), or exemestane (8%)."</t>
+  </si>
+  <si>
+    <t>1, 2, 3, 4, 5, 6, 7, 8, 792, 793, 794</t>
+  </si>
+  <si>
+    <t>trastuzumab emtansine</t>
+  </si>
+  <si>
+    <t>HER2+ breast cancer</t>
+  </si>
+  <si>
+    <t>This is the equivalent of https://dev.moalmanac.org/indications/ind:ema.kadcyla:0</t>
+  </si>
+  <si>
+    <t>pertuzumab with intravenous trastuzumab and chemotherapy</t>
+  </si>
+  <si>
+    <t>Split this row into 4 (see above 3 rows). I am fairly certain that this indication is the equivalent of this one: https://dev.moalmanac.org/indications/ind:ema.perjeta:1. The "Why the committee made these recommendations" section's first sentence adds "at high risk of recurrence" qualifier. Add "This indication is based on APHINITY (BO25126), a multicenter, randomized, double-blind, placebo-controlled phase 3 trial. Investigators selected one of the following chemotherapy regimes: (i) 3 or 4 cycles of FEC or 5-fluorouracil, doxorubicin and cyclophosphamide (FAC), followed by 3 or 4 cycles of docetaxel or 12 cycles of weekly paclitaxel; (ii) 4 cycles of AC or epirubicin and cyclophosphamide (EC), followed by 3 or 4 cycles of docetaxel or 12 cycles of weekly paclitaxel; or (iii) 6 cycles of docetaxel in combination with carboplatin." to the indication's description.</t>
+  </si>
+  <si>
+    <t>355, 356, 357, 358, 360</t>
+  </si>
+  <si>
+    <t>Midostaurin with daunorubicin and cytarabine</t>
+  </si>
+  <si>
+    <t>FLT3-mutation positive acute myeloid leukemia</t>
+  </si>
+  <si>
+    <t>This is the equivalent of https://dev.moalmanac.org/indications/ind:ema.rydapt:0. We only curated FLT3-ITD for the EMA because they don't have language detailing which variants qualify, whereas the FDA defers to their approved companion diagnostics. RYDAPT's companion diagnostic details several TKD variants, see here: https://dev.moalmanac.org/indications/ind:fda.rydapt:0. Adding just the FLT3-ITD proposition for now.</t>
+  </si>
+  <si>
+    <t>FLT3-mutation positive AML</t>
+  </si>
+  <si>
+    <t>This is the equivalent of https://dev.moalmanac.org/indications/ind:ema.xospata:0. We added FLT3 p.D835Y because the EMA product information specifically states that amino acid change. Adding only the FLT3-ITD proposition for now</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is rthe equivalent of https://dev.moalmanac.org/indications/ind:ema.vanflyta:0 </t>
+  </si>
+  <si>
+    <t>877, 878, 879</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unlike the EMA and FDA, this NICE approval does not detail what they specifically mean by RAS, at least from my reading. Let me know if you find any clarifyingn details! Assuming that NICE does not disambiguiate, I'd keep keep the first one as Wild type KRAS + Wild type KRAS + Wild type NRAS for the time being. This would be two indications (1.1 and 1.2), each with two propositions (FOLFOX and FOLFIRI). We only did Wild type KRAS + NRAS because that is what the EMA approval for panitumumab states. </t>
+  </si>
+  <si>
+    <t>556 (cetuximab + FOLFOX), will need to make a new proposition for cetuximab + FOLFIRI; 690, 691 (if you want to do KRAS + NRAS for panitumumab)</t>
+  </si>
+  <si>
+    <t>Propositions don't consider therapy line in moalmanac</t>
+  </si>
+  <si>
+    <t>169, 507</t>
+  </si>
+  <si>
+    <t>"OR" conditions as treated as separate propositions. Here is the equivalent EMA approval: https://dev.moalmanac.org/indications/ind:ema.tecentriq:4</t>
+  </si>
+  <si>
+    <t>672, 678</t>
+  </si>
+  <si>
+    <t>TA683</t>
+  </si>
+  <si>
+    <t>TA724</t>
+  </si>
+  <si>
+    <t>TA865</t>
+  </si>
+  <si>
+    <t>TA208</t>
+  </si>
+  <si>
+    <t>This is an OR statement of (capecitabine and cisplatin) OR (cisplatin and fluorouracil). The equivalent EMA approval is here: https://dev.moalmanac.org/indications/ind:ema.herceptin:8</t>
+  </si>
+  <si>
+    <t>570, 571</t>
+  </si>
+  <si>
+    <t>pembrolizumab + pemetrexed + platinum based chemotherapy</t>
+  </si>
+  <si>
+    <t>NSCLC</t>
+  </si>
+  <si>
+    <t>Here is the equivalent EMA approval: https://dev.moalmanac.org/indications/ind:ema.keytruda:1. Add "This indication is based on results from KEYNOTE-024, where patients received pembrolizumab in combination with investigator's choice of platinum-containing chemotherapy, including: pemetrexed with carboplatin, pemetrexed with cisplatin, gemcitabine and cisplatin, gemcitabine and carboplatin, or paclitaxel and carboplatin." to the indication's description.</t>
+  </si>
+  <si>
+    <t>316, 317, 592, 593, 594</t>
+  </si>
+  <si>
+    <t>Nivolumab + ipilimumab + chemotherapy</t>
+  </si>
+  <si>
+    <t>Here is the equivalent EMA approval: https://dev.moalmanac.org/indications/ind:ema.opdivo:0. Add "This indication is based on CA2099LA, a phase 3, randomized, and open-label study in which the platinum-based chemotherapy was either carboplatin and pemetrexed or cisplatin and pemetrexed for non-squamous NSCLC, or carboplatin and paclitaxel for squamous NSCLC." to the indication's description.</t>
+  </si>
+  <si>
+    <t>173, 174, 175</t>
+  </si>
+  <si>
+    <t>nivolumab + fluoropyrimidine and platinum-based chemotherapy</t>
+  </si>
+  <si>
+    <t>osephageal squamous cell carcinoma</t>
+  </si>
+  <si>
+    <t>Here is the equivalent EMA approval: https://dev.moalmanac.org/indications/ind:ema.opdivo:5. Add "This indication is based on CA209648, a randomized, active-controlled, and open-label study where the choice of chemotherapy was fluorouracil and cisplatin." to the indication's description.</t>
   </si>
 </sst>
 </file>
@@ -1255,7 +1390,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1289,12 +1424,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1380,6 +1524,9 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1387,8 +1534,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1703,20 +1853,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
     </row>
     <row r="2" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
+      <c r="B2" s="37"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -1809,7 +1959,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1910,7 +2060,7 @@
       <c r="H3" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I3" s="38" t="s">
+      <c r="I3" s="35" t="s">
         <v>350</v>
       </c>
     </row>
@@ -2224,7 +2374,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>84</v>
+        <v>400</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>85</v>
@@ -2244,886 +2394,866 @@
       <c r="H14" s="18" t="s">
         <v>28</v>
       </c>
+      <c r="I14" s="33" t="s">
+        <v>401</v>
+      </c>
+      <c r="J14" t="s">
+        <v>402</v>
+      </c>
     </row>
     <row r="15" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="19">
+      <c r="A15" s="15"/>
+      <c r="B15" s="16" t="s">
+        <v>397</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>403</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>404</v>
+      </c>
+      <c r="E15" s="22"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="33" t="s">
+        <v>405</v>
+      </c>
+      <c r="J15" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="15"/>
+      <c r="B16" s="16" t="s">
+        <v>398</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>407</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>404</v>
+      </c>
+      <c r="E16" s="22"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="33" t="s">
+        <v>408</v>
+      </c>
+      <c r="J16" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="15"/>
+      <c r="B17" s="16" t="s">
+        <v>399</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>410</v>
+      </c>
+      <c r="D17" s="16" t="s">
+        <v>411</v>
+      </c>
+      <c r="E17" s="22"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="33" t="s">
+        <v>412</v>
+      </c>
+      <c r="J17">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="19">
         <v>14</v>
       </c>
-      <c r="B15" s="20" t="s">
+      <c r="B18" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="C15" s="20" t="s">
+      <c r="C18" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="D15" s="20" t="s">
+      <c r="D18" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="E15" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F15" s="20" t="s">
+      <c r="E18" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F18" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G15" s="20" t="s">
+      <c r="G18" s="20" t="s">
         <v>93</v>
       </c>
-      <c r="H15" s="21" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="15">
+      <c r="H18" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="I18" s="40" t="s">
+        <v>395</v>
+      </c>
+      <c r="J18" s="40" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="15">
         <v>15</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B19" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C19" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="D16" s="16" t="s">
+      <c r="D19" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="E16" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F16" s="16" t="s">
+      <c r="E19" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F19" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="G16" s="16" t="s">
+      <c r="G19" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="H16" s="18" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="19">
+      <c r="H19" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="I19" s="40" t="s">
+        <v>393</v>
+      </c>
+      <c r="J19" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="19">
         <v>16</v>
       </c>
-      <c r="B17" s="20" t="s">
+      <c r="B20" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="C17" s="20" t="s">
+      <c r="C20" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="D17" s="20" t="s">
+      <c r="D20" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="E17" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F17" s="20" t="s">
+      <c r="E20" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F20" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="G17" s="20" t="s">
+      <c r="G20" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="H17" s="21" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="15">
+      <c r="H20" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="I20" s="33" t="s">
+        <v>391</v>
+      </c>
+      <c r="J20" s="33" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="15">
         <v>17</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B21" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="C21" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="D18" s="16" t="s">
+      <c r="D21" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="E18" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F18" s="16" t="s">
+      <c r="E21" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F21" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="G18" s="16" t="s">
+      <c r="G21" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="H18" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="I18" s="34" t="s">
+      <c r="H21" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="I21" s="34" t="s">
         <v>367</v>
       </c>
-      <c r="J18" s="34" t="s">
+      <c r="J21" s="34" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="19">
+    <row r="22" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="15"/>
+      <c r="B22" s="16" t="s">
+        <v>234</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>384</v>
+      </c>
+      <c r="D22" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="E22" s="22"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="39" t="s">
+        <v>386</v>
+      </c>
+      <c r="J22" s="39">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="15"/>
+      <c r="B23" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>202</v>
+      </c>
+      <c r="D23" s="16" t="s">
+        <v>387</v>
+      </c>
+      <c r="E23" s="22"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="39" t="s">
+        <v>388</v>
+      </c>
+      <c r="J23" s="39">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="19">
         <v>18</v>
       </c>
-      <c r="B19" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>108</v>
-      </c>
-      <c r="D19" s="20" t="s">
+      <c r="B24" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="C24" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="D24" s="20" t="s">
         <v>109</v>
       </c>
-      <c r="E19" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F19" s="20" t="s">
+      <c r="E24" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F24" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="G19" s="20" t="s">
+      <c r="G24" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="H19" s="21" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="15">
-        <v>19</v>
-      </c>
-      <c r="B20" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="D20" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="E20" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F20" s="16" t="s">
-        <v>115</v>
-      </c>
-      <c r="G20" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="H20" s="18" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="19">
+      <c r="H24" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="I24" s="39" t="s">
+        <v>389</v>
+      </c>
+      <c r="J24" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="19"/>
+      <c r="B25" s="20" t="s">
+        <v>368</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>371</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>372</v>
+      </c>
+      <c r="E25" s="22"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="21"/>
+      <c r="I25" t="s">
+        <v>373</v>
+      </c>
+      <c r="J25" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="19"/>
+      <c r="B26" s="20" t="s">
+        <v>283</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>375</v>
+      </c>
+      <c r="D26" s="20" t="s">
+        <v>372</v>
+      </c>
+      <c r="E26" s="22"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="21"/>
+      <c r="I26" t="s">
+        <v>376</v>
+      </c>
+      <c r="J26" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="19"/>
+      <c r="B27" s="20" t="s">
+        <v>369</v>
+      </c>
+      <c r="C27" s="20" t="s">
+        <v>378</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>379</v>
+      </c>
+      <c r="E27" s="22"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="21"/>
+      <c r="I27" t="s">
+        <v>380</v>
+      </c>
+      <c r="J27">
         <v>20</v>
-      </c>
-      <c r="B21" s="20" t="s">
-        <v>366</v>
-      </c>
-      <c r="C21" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="D21" s="20" t="s">
-        <v>119</v>
-      </c>
-      <c r="E21" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F21" s="20" t="s">
-        <v>120</v>
-      </c>
-      <c r="G21" s="20" t="s">
-        <v>121</v>
-      </c>
-      <c r="H21" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="I21" s="33" t="s">
-        <v>365</v>
-      </c>
-      <c r="J21" s="33" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="15">
-        <v>21</v>
-      </c>
-      <c r="B22" s="16" t="s">
-        <v>122</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>123</v>
-      </c>
-      <c r="D22" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="E22" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F22" s="16" t="s">
-        <v>125</v>
-      </c>
-      <c r="G22" s="16" t="s">
-        <v>126</v>
-      </c>
-      <c r="H22" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="I22" s="34" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="19">
-        <v>22</v>
-      </c>
-      <c r="B23" s="20" t="s">
-        <v>127</v>
-      </c>
-      <c r="C23" s="20" t="s">
-        <v>128</v>
-      </c>
-      <c r="D23" s="20" t="s">
-        <v>129</v>
-      </c>
-      <c r="E23" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F23" s="20" t="s">
-        <v>130</v>
-      </c>
-      <c r="G23" s="20" t="s">
-        <v>131</v>
-      </c>
-      <c r="H23" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="I23" s="33" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="15">
-        <v>23</v>
-      </c>
-      <c r="B24" s="16" t="s">
-        <v>132</v>
-      </c>
-      <c r="C24" s="16" t="s">
-        <v>133</v>
-      </c>
-      <c r="D24" s="16" t="s">
-        <v>134</v>
-      </c>
-      <c r="E24" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F24" s="16" t="s">
-        <v>135</v>
-      </c>
-      <c r="G24" s="16" t="s">
-        <v>136</v>
-      </c>
-      <c r="H24" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="I24" s="34" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="19">
-        <v>24</v>
-      </c>
-      <c r="B25" s="20" t="s">
-        <v>137</v>
-      </c>
-      <c r="C25" s="20" t="s">
-        <v>138</v>
-      </c>
-      <c r="D25" s="20" t="s">
-        <v>139</v>
-      </c>
-      <c r="E25" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F25" s="20" t="s">
-        <v>140</v>
-      </c>
-      <c r="G25" s="20" t="s">
-        <v>141</v>
-      </c>
-      <c r="H25" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="I25" s="33" t="s">
-        <v>360</v>
-      </c>
-      <c r="J25" s="33" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="15">
-        <v>25</v>
-      </c>
-      <c r="B26" s="16" t="s">
-        <v>142</v>
-      </c>
-      <c r="C26" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="D26" s="16" t="s">
-        <v>144</v>
-      </c>
-      <c r="E26" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F26" s="16" t="s">
-        <v>145</v>
-      </c>
-      <c r="G26" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="H26" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="I26" s="34" t="s">
-        <v>358</v>
-      </c>
-      <c r="J26" s="34" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="19">
-        <v>26</v>
-      </c>
-      <c r="B27" s="20" t="s">
-        <v>147</v>
-      </c>
-      <c r="C27" s="20" t="s">
-        <v>148</v>
-      </c>
-      <c r="D27" s="20" t="s">
-        <v>149</v>
-      </c>
-      <c r="E27" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F27" s="20" t="s">
-        <v>150</v>
-      </c>
-      <c r="G27" s="20" t="s">
-        <v>151</v>
-      </c>
-      <c r="H27" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="I27" s="33" t="s">
-        <v>357</v>
-      </c>
-      <c r="J27">
-        <v>641</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="15">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>152</v>
+        <v>370</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>90</v>
+        <v>381</v>
       </c>
       <c r="D28" s="16" t="s">
-        <v>153</v>
+        <v>379</v>
       </c>
       <c r="E28" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F28" s="16" t="s">
-        <v>154</v>
+        <v>115</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>155</v>
+        <v>116</v>
       </c>
       <c r="H28" s="18" t="s">
         <v>28</v>
       </c>
       <c r="I28" s="34" t="s">
-        <v>356</v>
-      </c>
-      <c r="J28">
-        <v>671</v>
+        <v>382</v>
+      </c>
+      <c r="J28" s="34" t="s">
+        <v>383</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="19">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>156</v>
+        <v>366</v>
       </c>
       <c r="C29" s="20" t="s">
-        <v>157</v>
+        <v>118</v>
       </c>
       <c r="D29" s="20" t="s">
-        <v>158</v>
+        <v>119</v>
       </c>
       <c r="E29" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F29" s="20" t="s">
-        <v>159</v>
+        <v>120</v>
       </c>
       <c r="G29" s="20" t="s">
-        <v>160</v>
+        <v>121</v>
       </c>
       <c r="H29" s="21" t="s">
         <v>28</v>
       </c>
       <c r="I29" s="33" t="s">
-        <v>354</v>
+        <v>365</v>
       </c>
       <c r="J29" s="33" t="s">
-        <v>355</v>
+        <v>364</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="15">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>161</v>
+        <v>122</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>162</v>
+        <v>123</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>163</v>
+        <v>124</v>
       </c>
       <c r="E30" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F30" s="16" t="s">
-        <v>164</v>
+        <v>125</v>
       </c>
       <c r="G30" s="16" t="s">
-        <v>165</v>
+        <v>126</v>
       </c>
       <c r="H30" s="18" t="s">
         <v>28</v>
       </c>
       <c r="I30" s="34" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="19">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>166</v>
+        <v>127</v>
       </c>
       <c r="C31" s="20" t="s">
-        <v>167</v>
+        <v>128</v>
       </c>
       <c r="D31" s="20" t="s">
-        <v>168</v>
+        <v>129</v>
       </c>
       <c r="E31" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F31" s="20" t="s">
-        <v>169</v>
+        <v>130</v>
       </c>
       <c r="G31" s="20" t="s">
-        <v>170</v>
+        <v>131</v>
       </c>
       <c r="H31" s="21" t="s">
         <v>28</v>
       </c>
       <c r="I31" s="33" t="s">
-        <v>339</v>
+        <v>363</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="15">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>171</v>
+        <v>132</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>172</v>
+        <v>133</v>
       </c>
       <c r="D32" s="16" t="s">
-        <v>173</v>
+        <v>134</v>
       </c>
       <c r="E32" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F32" s="16" t="s">
-        <v>174</v>
+        <v>135</v>
       </c>
       <c r="G32" s="16" t="s">
-        <v>175</v>
+        <v>136</v>
       </c>
       <c r="H32" s="18" t="s">
         <v>28</v>
       </c>
       <c r="I32" s="34" t="s">
-        <v>338</v>
+        <v>362</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="19">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>176</v>
+        <v>137</v>
       </c>
       <c r="C33" s="20" t="s">
-        <v>177</v>
+        <v>138</v>
       </c>
       <c r="D33" s="20" t="s">
-        <v>178</v>
+        <v>139</v>
       </c>
       <c r="E33" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F33" s="20" t="s">
-        <v>179</v>
+        <v>140</v>
       </c>
       <c r="G33" s="20" t="s">
-        <v>180</v>
+        <v>141</v>
       </c>
       <c r="H33" s="21" t="s">
         <v>28</v>
       </c>
       <c r="I33" s="33" t="s">
-        <v>337</v>
+        <v>360</v>
+      </c>
+      <c r="J33" s="33" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="15">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>181</v>
+        <v>142</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>182</v>
+        <v>143</v>
       </c>
       <c r="D34" s="16" t="s">
-        <v>183</v>
+        <v>144</v>
       </c>
       <c r="E34" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F34" s="16" t="s">
-        <v>184</v>
+        <v>145</v>
       </c>
       <c r="G34" s="16" t="s">
-        <v>185</v>
+        <v>146</v>
       </c>
       <c r="H34" s="18" t="s">
         <v>28</v>
       </c>
       <c r="I34" s="34" t="s">
-        <v>336</v>
+        <v>358</v>
+      </c>
+      <c r="J34" s="34" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="19">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>186</v>
+        <v>147</v>
       </c>
       <c r="C35" s="20" t="s">
-        <v>187</v>
+        <v>148</v>
       </c>
       <c r="D35" s="20" t="s">
-        <v>188</v>
-      </c>
-      <c r="E35" s="23" t="s">
-        <v>9</v>
+        <v>149</v>
+      </c>
+      <c r="E35" s="22" t="s">
+        <v>7</v>
       </c>
       <c r="F35" s="20" t="s">
-        <v>189</v>
+        <v>150</v>
       </c>
       <c r="G35" s="20" t="s">
-        <v>190</v>
+        <v>151</v>
       </c>
       <c r="H35" s="21" t="s">
         <v>28</v>
       </c>
       <c r="I35" s="33" t="s">
-        <v>335</v>
+        <v>357</v>
+      </c>
+      <c r="J35">
+        <v>641</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="15">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>191</v>
+        <v>152</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>192</v>
+        <v>90</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>193</v>
-      </c>
-      <c r="E36" s="24" t="s">
-        <v>11</v>
+        <v>153</v>
+      </c>
+      <c r="E36" s="22" t="s">
+        <v>7</v>
       </c>
       <c r="F36" s="16" t="s">
-        <v>194</v>
+        <v>154</v>
       </c>
       <c r="G36" s="16" t="s">
-        <v>195</v>
+        <v>155</v>
       </c>
       <c r="H36" s="18" t="s">
         <v>28</v>
       </c>
       <c r="I36" s="34" t="s">
-        <v>334</v>
+        <v>356</v>
+      </c>
+      <c r="J36">
+        <v>671</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="19">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>196</v>
+        <v>156</v>
       </c>
       <c r="C37" s="20" t="s">
-        <v>197</v>
+        <v>157</v>
       </c>
       <c r="D37" s="20" t="s">
-        <v>198</v>
-      </c>
-      <c r="E37" s="24" t="s">
-        <v>11</v>
+        <v>158</v>
+      </c>
+      <c r="E37" s="22" t="s">
+        <v>7</v>
       </c>
       <c r="F37" s="20" t="s">
-        <v>199</v>
+        <v>159</v>
       </c>
       <c r="G37" s="20" t="s">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="H37" s="21" t="s">
         <v>28</v>
       </c>
       <c r="I37" s="33" t="s">
-        <v>333</v>
+        <v>354</v>
+      </c>
+      <c r="J37" s="33" t="s">
+        <v>355</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="15">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>201</v>
+        <v>161</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>202</v>
+        <v>162</v>
       </c>
       <c r="D38" s="16" t="s">
-        <v>203</v>
-      </c>
-      <c r="E38" s="24" t="s">
-        <v>11</v>
+        <v>163</v>
+      </c>
+      <c r="E38" s="22" t="s">
+        <v>7</v>
       </c>
       <c r="F38" s="16" t="s">
-        <v>204</v>
+        <v>164</v>
       </c>
       <c r="G38" s="16" t="s">
-        <v>205</v>
+        <v>165</v>
       </c>
       <c r="H38" s="18" t="s">
         <v>28</v>
       </c>
       <c r="I38" s="34" t="s">
-        <v>332</v>
+        <v>353</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="19">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>206</v>
+        <v>166</v>
       </c>
       <c r="C39" s="20" t="s">
-        <v>207</v>
+        <v>167</v>
       </c>
       <c r="D39" s="20" t="s">
-        <v>208</v>
-      </c>
-      <c r="E39" s="25" t="s">
-        <v>13</v>
+        <v>168</v>
+      </c>
+      <c r="E39" s="22" t="s">
+        <v>7</v>
       </c>
       <c r="F39" s="20" t="s">
-        <v>209</v>
+        <v>169</v>
       </c>
       <c r="G39" s="20" t="s">
-        <v>210</v>
+        <v>170</v>
       </c>
       <c r="H39" s="21" t="s">
         <v>28</v>
       </c>
       <c r="I39" s="33" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="15">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>211</v>
+        <v>171</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>207</v>
+        <v>172</v>
       </c>
       <c r="D40" s="16" t="s">
-        <v>212</v>
-      </c>
-      <c r="E40" s="25" t="s">
-        <v>13</v>
+        <v>173</v>
+      </c>
+      <c r="E40" s="22" t="s">
+        <v>7</v>
       </c>
       <c r="F40" s="16" t="s">
-        <v>213</v>
+        <v>174</v>
       </c>
       <c r="G40" s="16" t="s">
-        <v>214</v>
+        <v>175</v>
       </c>
       <c r="H40" s="18" t="s">
         <v>28</v>
       </c>
       <c r="I40" s="34" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="19">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>215</v>
+        <v>176</v>
       </c>
       <c r="C41" s="20" t="s">
-        <v>216</v>
+        <v>177</v>
       </c>
       <c r="D41" s="20" t="s">
-        <v>217</v>
-      </c>
-      <c r="E41" s="25" t="s">
-        <v>13</v>
+        <v>178</v>
+      </c>
+      <c r="E41" s="22" t="s">
+        <v>7</v>
       </c>
       <c r="F41" s="20" t="s">
-        <v>218</v>
+        <v>179</v>
       </c>
       <c r="G41" s="20" t="s">
-        <v>219</v>
+        <v>180</v>
       </c>
       <c r="H41" s="21" t="s">
         <v>28</v>
       </c>
       <c r="I41" s="33" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="15">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>220</v>
+        <v>181</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>207</v>
+        <v>182</v>
       </c>
       <c r="D42" s="16" t="s">
-        <v>221</v>
-      </c>
-      <c r="E42" s="25" t="s">
-        <v>13</v>
+        <v>183</v>
+      </c>
+      <c r="E42" s="22" t="s">
+        <v>7</v>
       </c>
       <c r="F42" s="16" t="s">
-        <v>222</v>
+        <v>184</v>
       </c>
       <c r="G42" s="16" t="s">
-        <v>223</v>
+        <v>185</v>
       </c>
       <c r="H42" s="18" t="s">
         <v>28</v>
       </c>
       <c r="I42" s="34" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="19">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>224</v>
+        <v>186</v>
       </c>
       <c r="C43" s="20" t="s">
-        <v>207</v>
+        <v>187</v>
       </c>
       <c r="D43" s="20" t="s">
-        <v>225</v>
-      </c>
-      <c r="E43" s="25" t="s">
-        <v>13</v>
+        <v>188</v>
+      </c>
+      <c r="E43" s="23" t="s">
+        <v>9</v>
       </c>
       <c r="F43" s="20" t="s">
-        <v>226</v>
+        <v>189</v>
       </c>
       <c r="G43" s="20" t="s">
-        <v>227</v>
+        <v>190</v>
       </c>
       <c r="H43" s="21" t="s">
         <v>28</v>
       </c>
       <c r="I43" s="33" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="15">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>228</v>
-      </c>
-      <c r="E44" s="25" t="s">
-        <v>13</v>
+        <v>193</v>
+      </c>
+      <c r="E44" s="24" t="s">
+        <v>11</v>
       </c>
       <c r="F44" s="16" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="G44" s="16" t="s">
-        <v>230</v>
+        <v>195</v>
       </c>
       <c r="H44" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="I44" t="s">
-        <v>326</v>
+      <c r="I44" s="34" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="19">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="B45" s="20" t="s">
         <v>196</v>
@@ -3132,503 +3262,735 @@
         <v>197</v>
       </c>
       <c r="D45" s="20" t="s">
-        <v>231</v>
-      </c>
-      <c r="E45" s="25" t="s">
-        <v>13</v>
+        <v>198</v>
+      </c>
+      <c r="E45" s="24" t="s">
+        <v>11</v>
       </c>
       <c r="F45" s="20" t="s">
-        <v>232</v>
+        <v>199</v>
       </c>
       <c r="G45" s="20" t="s">
-        <v>233</v>
+        <v>200</v>
       </c>
       <c r="H45" s="21" t="s">
         <v>28</v>
       </c>
       <c r="I45" s="33" t="s">
-        <v>324</v>
-      </c>
-      <c r="J45" s="33" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="15">
-        <v>45</v>
-      </c>
-      <c r="B46" s="26" t="s">
-        <v>234</v>
-      </c>
-      <c r="C46" s="26" t="s">
-        <v>235</v>
-      </c>
-      <c r="D46" s="26" t="s">
-        <v>236</v>
-      </c>
-      <c r="E46" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="F46" s="26" t="s">
-        <v>237</v>
-      </c>
-      <c r="G46" s="26" t="s">
-        <v>238</v>
+        <v>37</v>
+      </c>
+      <c r="B46" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="C46" s="16" t="s">
+        <v>202</v>
+      </c>
+      <c r="D46" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="E46" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F46" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="G46" s="16" t="s">
+        <v>205</v>
       </c>
       <c r="H46" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="I46" s="30" t="s">
-        <v>323</v>
+      <c r="I46" s="34" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="19">
-        <v>46</v>
-      </c>
-      <c r="B47" s="27" t="s">
-        <v>239</v>
-      </c>
-      <c r="C47" s="27" t="s">
-        <v>177</v>
-      </c>
-      <c r="D47" s="27" t="s">
-        <v>240</v>
-      </c>
-      <c r="E47" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="F47" s="27" t="s">
-        <v>241</v>
-      </c>
-      <c r="G47" s="27" t="s">
-        <v>242</v>
+        <v>38</v>
+      </c>
+      <c r="B47" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="C47" s="20" t="s">
+        <v>207</v>
+      </c>
+      <c r="D47" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="E47" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47" s="20" t="s">
+        <v>209</v>
+      </c>
+      <c r="G47" s="20" t="s">
+        <v>210</v>
       </c>
       <c r="H47" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I47" s="31" t="s">
-        <v>322</v>
+      <c r="I47" s="33" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="15">
-        <v>47</v>
-      </c>
-      <c r="B48" s="26" t="s">
-        <v>239</v>
-      </c>
-      <c r="C48" s="26" t="s">
-        <v>177</v>
-      </c>
-      <c r="D48" s="26" t="s">
-        <v>243</v>
-      </c>
-      <c r="E48" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F48" s="26" t="s">
-        <v>244</v>
-      </c>
-      <c r="G48" s="26" t="s">
-        <v>245</v>
+        <v>39</v>
+      </c>
+      <c r="B48" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="C48" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="D48" s="16" t="s">
+        <v>212</v>
+      </c>
+      <c r="E48" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F48" s="16" t="s">
+        <v>213</v>
+      </c>
+      <c r="G48" s="16" t="s">
+        <v>214</v>
       </c>
       <c r="H48" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="I48" s="30" t="s">
-        <v>321</v>
+      <c r="I48" s="34" t="s">
+        <v>330</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="19">
-        <v>48</v>
-      </c>
-      <c r="B49" s="27" t="s">
-        <v>246</v>
-      </c>
-      <c r="C49" s="27" t="s">
-        <v>247</v>
-      </c>
-      <c r="D49" s="27" t="s">
-        <v>248</v>
-      </c>
-      <c r="E49" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F49" s="27" t="s">
-        <v>249</v>
-      </c>
-      <c r="G49" s="27" t="s">
-        <v>250</v>
+        <v>40</v>
+      </c>
+      <c r="B49" s="20" t="s">
+        <v>215</v>
+      </c>
+      <c r="C49" s="20" t="s">
+        <v>216</v>
+      </c>
+      <c r="D49" s="20" t="s">
+        <v>217</v>
+      </c>
+      <c r="E49" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F49" s="20" t="s">
+        <v>218</v>
+      </c>
+      <c r="G49" s="20" t="s">
+        <v>219</v>
       </c>
       <c r="H49" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I49" s="31" t="s">
-        <v>320</v>
+      <c r="I49" s="33" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="15">
-        <v>49</v>
-      </c>
-      <c r="B50" s="26" t="s">
-        <v>251</v>
-      </c>
-      <c r="C50" s="26" t="s">
-        <v>252</v>
-      </c>
-      <c r="D50" s="26" t="s">
-        <v>253</v>
-      </c>
-      <c r="E50" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F50" s="26" t="s">
-        <v>254</v>
-      </c>
-      <c r="G50" s="26" t="s">
-        <v>255</v>
+        <v>41</v>
+      </c>
+      <c r="B50" s="16" t="s">
+        <v>220</v>
+      </c>
+      <c r="C50" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="D50" s="16" t="s">
+        <v>221</v>
+      </c>
+      <c r="E50" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F50" s="16" t="s">
+        <v>222</v>
+      </c>
+      <c r="G50" s="16" t="s">
+        <v>223</v>
       </c>
       <c r="H50" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="I50" s="30" t="s">
-        <v>309</v>
+      <c r="I50" s="34" t="s">
+        <v>328</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="19">
-        <v>50</v>
-      </c>
-      <c r="B51" s="27" t="s">
-        <v>69</v>
-      </c>
-      <c r="C51" s="27" t="s">
-        <v>256</v>
-      </c>
-      <c r="D51" s="27" t="s">
-        <v>257</v>
-      </c>
-      <c r="E51" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F51" s="27" t="s">
-        <v>258</v>
-      </c>
-      <c r="G51" s="27" t="s">
-        <v>259</v>
+        <v>42</v>
+      </c>
+      <c r="B51" s="20" t="s">
+        <v>224</v>
+      </c>
+      <c r="C51" s="20" t="s">
+        <v>207</v>
+      </c>
+      <c r="D51" s="20" t="s">
+        <v>225</v>
+      </c>
+      <c r="E51" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F51" s="20" t="s">
+        <v>226</v>
+      </c>
+      <c r="G51" s="20" t="s">
+        <v>227</v>
       </c>
       <c r="H51" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I51" s="31" t="s">
-        <v>311</v>
-      </c>
-      <c r="J51" s="31" t="s">
-        <v>312</v>
+      <c r="I51" s="33" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="15">
-        <v>51</v>
-      </c>
-      <c r="B52" s="26" t="s">
-        <v>260</v>
-      </c>
-      <c r="C52" s="26" t="s">
-        <v>261</v>
-      </c>
-      <c r="D52" s="26" t="s">
-        <v>262</v>
-      </c>
-      <c r="E52" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F52" s="26" t="s">
-        <v>263</v>
-      </c>
-      <c r="G52" s="26" t="s">
-        <v>264</v>
+        <v>43</v>
+      </c>
+      <c r="B52" s="16" t="s">
+        <v>186</v>
+      </c>
+      <c r="C52" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="D52" s="16" t="s">
+        <v>228</v>
+      </c>
+      <c r="E52" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F52" s="16" t="s">
+        <v>229</v>
+      </c>
+      <c r="G52" s="16" t="s">
+        <v>230</v>
       </c>
       <c r="H52" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="I52" s="30" t="s">
-        <v>318</v>
-      </c>
-      <c r="J52" s="30" t="s">
-        <v>319</v>
+      <c r="I52" t="s">
+        <v>326</v>
       </c>
     </row>
     <row r="53" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="19">
-        <v>52</v>
-      </c>
-      <c r="B53" s="27" t="s">
-        <v>265</v>
-      </c>
-      <c r="C53" s="27" t="s">
-        <v>266</v>
-      </c>
-      <c r="D53" s="27" t="s">
-        <v>183</v>
-      </c>
-      <c r="E53" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F53" s="27" t="s">
-        <v>267</v>
-      </c>
-      <c r="G53" s="27" t="s">
-        <v>268</v>
+        <v>44</v>
+      </c>
+      <c r="B53" s="20" t="s">
+        <v>196</v>
+      </c>
+      <c r="C53" s="20" t="s">
+        <v>197</v>
+      </c>
+      <c r="D53" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="E53" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F53" s="20" t="s">
+        <v>232</v>
+      </c>
+      <c r="G53" s="20" t="s">
+        <v>233</v>
       </c>
       <c r="H53" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I53" s="31" t="s">
-        <v>316</v>
-      </c>
-      <c r="J53" s="31" t="s">
-        <v>317</v>
+      <c r="I53" s="33" t="s">
+        <v>324</v>
+      </c>
+      <c r="J53" s="33" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="15">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="B54" s="26" t="s">
-        <v>269</v>
+        <v>234</v>
       </c>
       <c r="C54" s="26" t="s">
-        <v>207</v>
+        <v>235</v>
       </c>
       <c r="D54" s="26" t="s">
-        <v>270</v>
-      </c>
-      <c r="E54" s="22" t="s">
-        <v>7</v>
+        <v>236</v>
+      </c>
+      <c r="E54" s="17" t="s">
+        <v>5</v>
       </c>
       <c r="F54" s="26" t="s">
-        <v>271</v>
+        <v>237</v>
       </c>
       <c r="G54" s="26" t="s">
-        <v>272</v>
+        <v>238</v>
       </c>
       <c r="H54" s="18" t="s">
         <v>28</v>
       </c>
       <c r="I54" s="30" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
     </row>
     <row r="55" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="19">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="B55" s="27" t="s">
-        <v>273</v>
+        <v>239</v>
       </c>
       <c r="C55" s="27" t="s">
-        <v>207</v>
+        <v>177</v>
       </c>
       <c r="D55" s="27" t="s">
-        <v>274</v>
-      </c>
-      <c r="E55" s="22" t="s">
-        <v>7</v>
+        <v>240</v>
+      </c>
+      <c r="E55" s="17" t="s">
+        <v>5</v>
       </c>
       <c r="F55" s="27" t="s">
-        <v>275</v>
+        <v>241</v>
       </c>
       <c r="G55" s="27" t="s">
-        <v>276</v>
+        <v>242</v>
       </c>
       <c r="H55" s="21" t="s">
         <v>28</v>
       </c>
       <c r="I55" s="31" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
     </row>
     <row r="56" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="15">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="B56" s="26" t="s">
-        <v>273</v>
+        <v>239</v>
       </c>
       <c r="C56" s="26" t="s">
-        <v>207</v>
+        <v>177</v>
       </c>
       <c r="D56" s="26" t="s">
-        <v>277</v>
+        <v>243</v>
       </c>
       <c r="E56" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F56" s="26" t="s">
-        <v>278</v>
+        <v>244</v>
       </c>
       <c r="G56" s="26" t="s">
-        <v>279</v>
+        <v>245</v>
       </c>
       <c r="H56" s="18" t="s">
         <v>28</v>
       </c>
       <c r="I56" s="30" t="s">
-        <v>310</v>
+        <v>321</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="19">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="B57" s="27" t="s">
-        <v>273</v>
+        <v>246</v>
       </c>
       <c r="C57" s="27" t="s">
-        <v>207</v>
+        <v>247</v>
       </c>
       <c r="D57" s="27" t="s">
-        <v>280</v>
+        <v>248</v>
       </c>
       <c r="E57" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F57" s="27" t="s">
-        <v>281</v>
+        <v>249</v>
       </c>
       <c r="G57" s="27" t="s">
-        <v>282</v>
+        <v>250</v>
       </c>
       <c r="H57" s="21" t="s">
         <v>28</v>
       </c>
       <c r="I57" s="31" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="15">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="B58" s="26" t="s">
-        <v>283</v>
+        <v>251</v>
       </c>
       <c r="C58" s="26" t="s">
-        <v>284</v>
+        <v>252</v>
       </c>
       <c r="D58" s="26" t="s">
-        <v>285</v>
+        <v>253</v>
       </c>
       <c r="E58" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F58" s="26" t="s">
-        <v>286</v>
+        <v>254</v>
       </c>
       <c r="G58" s="26" t="s">
-        <v>287</v>
+        <v>255</v>
       </c>
       <c r="H58" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="I58" s="32" t="s">
-        <v>307</v>
-      </c>
-      <c r="J58" t="s">
-        <v>308</v>
+      <c r="I58" s="30" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="19">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B59" s="27" t="s">
-        <v>288</v>
+        <v>69</v>
       </c>
       <c r="C59" s="27" t="s">
-        <v>207</v>
+        <v>256</v>
       </c>
       <c r="D59" s="27" t="s">
-        <v>289</v>
+        <v>257</v>
       </c>
       <c r="E59" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F59" s="27" t="s">
-        <v>290</v>
+        <v>258</v>
       </c>
       <c r="G59" s="27" t="s">
-        <v>291</v>
+        <v>259</v>
       </c>
       <c r="H59" s="21" t="s">
         <v>28</v>
       </c>
       <c r="I59" s="31" t="s">
-        <v>306</v>
+        <v>311</v>
+      </c>
+      <c r="J59" s="31" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="15">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="B60" s="26" t="s">
-        <v>292</v>
+        <v>260</v>
       </c>
       <c r="C60" s="26" t="s">
-        <v>157</v>
+        <v>261</v>
       </c>
       <c r="D60" s="26" t="s">
-        <v>293</v>
+        <v>262</v>
       </c>
       <c r="E60" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F60" s="26" t="s">
-        <v>294</v>
+        <v>263</v>
       </c>
       <c r="G60" s="26" t="s">
-        <v>295</v>
+        <v>264</v>
       </c>
       <c r="H60" s="18" t="s">
         <v>28</v>
       </c>
       <c r="I60" s="30" t="s">
-        <v>304</v>
+        <v>318</v>
       </c>
       <c r="J60" s="30" t="s">
-        <v>305</v>
+        <v>319</v>
       </c>
     </row>
     <row r="61" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="19">
+        <v>52</v>
+      </c>
+      <c r="B61" s="27" t="s">
+        <v>265</v>
+      </c>
+      <c r="C61" s="27" t="s">
+        <v>266</v>
+      </c>
+      <c r="D61" s="27" t="s">
+        <v>183</v>
+      </c>
+      <c r="E61" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F61" s="27" t="s">
+        <v>267</v>
+      </c>
+      <c r="G61" s="27" t="s">
+        <v>268</v>
+      </c>
+      <c r="H61" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="I61" s="31" t="s">
+        <v>316</v>
+      </c>
+      <c r="J61" s="31" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A62" s="15">
+        <v>53</v>
+      </c>
+      <c r="B62" s="26" t="s">
+        <v>269</v>
+      </c>
+      <c r="C62" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="D62" s="26" t="s">
+        <v>270</v>
+      </c>
+      <c r="E62" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F62" s="26" t="s">
+        <v>271</v>
+      </c>
+      <c r="G62" s="26" t="s">
+        <v>272</v>
+      </c>
+      <c r="H62" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="I62" s="30" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="19">
+        <v>54</v>
+      </c>
+      <c r="B63" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="C63" s="27" t="s">
+        <v>207</v>
+      </c>
+      <c r="D63" s="27" t="s">
+        <v>274</v>
+      </c>
+      <c r="E63" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F63" s="27" t="s">
+        <v>275</v>
+      </c>
+      <c r="G63" s="27" t="s">
+        <v>276</v>
+      </c>
+      <c r="H63" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="I63" s="31" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="15">
+        <v>55</v>
+      </c>
+      <c r="B64" s="26" t="s">
+        <v>273</v>
+      </c>
+      <c r="C64" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="D64" s="26" t="s">
+        <v>277</v>
+      </c>
+      <c r="E64" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F64" s="26" t="s">
+        <v>278</v>
+      </c>
+      <c r="G64" s="26" t="s">
+        <v>279</v>
+      </c>
+      <c r="H64" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="I64" s="30" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="19">
+        <v>56</v>
+      </c>
+      <c r="B65" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="C65" s="27" t="s">
+        <v>207</v>
+      </c>
+      <c r="D65" s="27" t="s">
+        <v>280</v>
+      </c>
+      <c r="E65" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F65" s="27" t="s">
+        <v>281</v>
+      </c>
+      <c r="G65" s="27" t="s">
+        <v>282</v>
+      </c>
+      <c r="H65" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="I65" s="31" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="15">
+        <v>57</v>
+      </c>
+      <c r="B66" s="26" t="s">
+        <v>283</v>
+      </c>
+      <c r="C66" s="26" t="s">
+        <v>284</v>
+      </c>
+      <c r="D66" s="26" t="s">
+        <v>285</v>
+      </c>
+      <c r="E66" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F66" s="26" t="s">
+        <v>286</v>
+      </c>
+      <c r="G66" s="26" t="s">
+        <v>287</v>
+      </c>
+      <c r="H66" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="I66" s="32" t="s">
+        <v>307</v>
+      </c>
+      <c r="J66" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="19">
+        <v>58</v>
+      </c>
+      <c r="B67" s="27" t="s">
+        <v>288</v>
+      </c>
+      <c r="C67" s="27" t="s">
+        <v>207</v>
+      </c>
+      <c r="D67" s="27" t="s">
+        <v>289</v>
+      </c>
+      <c r="E67" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F67" s="27" t="s">
+        <v>290</v>
+      </c>
+      <c r="G67" s="27" t="s">
+        <v>291</v>
+      </c>
+      <c r="H67" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="I67" s="31" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="15">
+        <v>59</v>
+      </c>
+      <c r="B68" s="26" t="s">
+        <v>292</v>
+      </c>
+      <c r="C68" s="26" t="s">
+        <v>157</v>
+      </c>
+      <c r="D68" s="26" t="s">
+        <v>293</v>
+      </c>
+      <c r="E68" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F68" s="26" t="s">
+        <v>294</v>
+      </c>
+      <c r="G68" s="26" t="s">
+        <v>295</v>
+      </c>
+      <c r="H68" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="I68" s="30" t="s">
+        <v>304</v>
+      </c>
+      <c r="J68" s="30" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="19">
         <v>60</v>
       </c>
-      <c r="B61" s="27" t="s">
+      <c r="B69" s="27" t="s">
         <v>296</v>
       </c>
-      <c r="C61" s="27" t="s">
+      <c r="C69" s="27" t="s">
         <v>297</v>
       </c>
-      <c r="D61" s="27" t="s">
+      <c r="D69" s="27" t="s">
         <v>298</v>
       </c>
-      <c r="E61" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F61" s="27" t="s">
+      <c r="E69" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F69" s="27" t="s">
         <v>299</v>
       </c>
-      <c r="G61" s="27" t="s">
+      <c r="G69" s="27" t="s">
         <v>300</v>
       </c>
-      <c r="H61" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="I61" s="29" t="s">
+      <c r="H69" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="I69" s="29" t="s">
         <v>303</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added propositions for most
</commit_message>
<xml_diff>
--- a/escalation_tracker.xlsx
+++ b/escalation_tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brendan/GitHub/projects/moalmanac-db-hscni/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brendan/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{380BB488-14FF-8C4C-864A-B5AF958CE543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB2E7E87-1E7C-D742-A551-D71EF8E8032D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="220" yWindow="600" windowWidth="31400" windowHeight="19140" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -21,12 +21,15 @@
     <sheet name="Data Error" sheetId="6" r:id="rId6"/>
     <sheet name="Standing Rule" sheetId="7" r:id="rId7"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Escalations'!$A$1:$J$69</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1023" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="415">
   <si>
     <t>NI-MOAlmanac — Brendan Escalation Tracker</t>
   </si>
@@ -1078,10 +1081,6 @@
     <t>Will need to create new propositions</t>
   </si>
   <si>
-    <t>This is an odd one. I am inclined to curate it as PD-L1 (TPS) &gt;= 0%. What do you think? They write this section in "Why the committee made these recommendations" Pembrolizumab combination therapy meets NICE's criteria to be considered a life-
-extending treatment at the end of life in both PD-L1 tumour proportion score subgroups. The cost-effectiveness estimates in people whose tumours express PD-L1 with a tumour proportion score of 0% to 49% were within what NICE considers a good use of NHS resources. For people whose tumours have a PD-L1 tumour proportion score of 50% or more and who need an urgent clinical intervention (for example, because their cancer may cause major airway blockage), the cost-effectiveness estimates were not certain. However, they are likely to be within what NICE considers a good use of NHS resources, so pembrolizumab combination is recommended in both groups."</t>
-  </si>
-  <si>
     <t>This is the equivalent of this relationship: https://ie.moalmanac.org/indications/ind:ema.imfinzi:3</t>
   </si>
   <si>
@@ -1266,6 +1265,15 @@
   </si>
   <si>
     <t>Here is the equivalent EMA approval: https://dev.moalmanac.org/indications/ind:ema.opdivo:5. Add "This indication is based on CA209648, a randomized, active-controlled, and open-label study where the choice of chemotherapy was fluorouracil and cisplatin." to the indication's description.</t>
+  </si>
+  <si>
+    <t>This is an odd one. I am inclined to curate it as PD-L1 (TPS) &gt;= 0%. What do you think? They write this section in "Why the committee made these recommendations" Pembrolizumab combination therapy meets NICE's criteria to be considered a life-extending treatment at the end of life in both PD-L1 tumour proportion score subgroups. The cost-effectiveness estimates in people whose tumours express PD-L1 with a tumour proportion score of 0% to 49% were within what NICE considers a good use of NHS resources. For people whose tumours have a PD-L1 tumour proportion score of 50% or more and who need an urgent clinical intervention (for example, because their cancer may cause major airway blockage), the cost-effectiveness estimates were not certain. However, they are likely to be within what NICE considers a good use of NHS resources, so pembrolizumab combination is recommended in both groups."</t>
+  </si>
+  <si>
+    <t>150, 151, 152, 153, 154, 155, 156, 157</t>
+  </si>
+  <si>
+    <t>327, 328</t>
   </si>
 </sst>
 </file>
@@ -1527,18 +1535,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1853,20 +1861,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
     </row>
     <row r="2" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -2034,6 +2042,9 @@
       <c r="I2" s="34" t="s">
         <v>349</v>
       </c>
+      <c r="J2">
+        <v>915</v>
+      </c>
     </row>
     <row r="3" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="19">
@@ -2061,7 +2072,10 @@
         <v>28</v>
       </c>
       <c r="I3" s="35" t="s">
-        <v>350</v>
+        <v>412</v>
+      </c>
+      <c r="J3">
+        <v>916</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -2092,6 +2106,9 @@
       <c r="I4" s="34" t="s">
         <v>349</v>
       </c>
+      <c r="J4">
+        <v>917</v>
+      </c>
     </row>
     <row r="5" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="19">
@@ -2121,6 +2138,9 @@
       <c r="I5" s="33" t="s">
         <v>345</v>
       </c>
+      <c r="J5">
+        <v>918</v>
+      </c>
     </row>
     <row r="6" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="15">
@@ -2270,10 +2290,10 @@
         <v>28</v>
       </c>
       <c r="I10" s="34" t="s">
+        <v>350</v>
+      </c>
+      <c r="J10" s="34" t="s">
         <v>351</v>
-      </c>
-      <c r="J10" s="34" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -2374,7 +2394,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>85</v>
@@ -2395,73 +2415,73 @@
         <v>28</v>
       </c>
       <c r="I14" s="33" t="s">
+        <v>400</v>
+      </c>
+      <c r="J14" t="s">
         <v>401</v>
-      </c>
-      <c r="J14" t="s">
-        <v>402</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="15"/>
       <c r="B15" s="16" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C15" s="16" t="s">
+        <v>402</v>
+      </c>
+      <c r="D15" s="16" t="s">
         <v>403</v>
-      </c>
-      <c r="D15" s="16" t="s">
-        <v>404</v>
       </c>
       <c r="E15" s="22"/>
       <c r="F15" s="16"/>
       <c r="G15" s="16"/>
       <c r="H15" s="18"/>
       <c r="I15" s="33" t="s">
+        <v>404</v>
+      </c>
+      <c r="J15" t="s">
         <v>405</v>
-      </c>
-      <c r="J15" t="s">
-        <v>406</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="15"/>
       <c r="B16" s="16" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E16" s="22"/>
       <c r="F16" s="16"/>
       <c r="G16" s="16"/>
       <c r="H16" s="18"/>
       <c r="I16" s="33" t="s">
+        <v>407</v>
+      </c>
+      <c r="J16" t="s">
         <v>408</v>
-      </c>
-      <c r="J16" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="15"/>
       <c r="B17" s="16" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C17" s="16" t="s">
+        <v>409</v>
+      </c>
+      <c r="D17" s="16" t="s">
         <v>410</v>
-      </c>
-      <c r="D17" s="16" t="s">
-        <v>411</v>
       </c>
       <c r="E17" s="22"/>
       <c r="F17" s="16"/>
       <c r="G17" s="16"/>
       <c r="H17" s="18"/>
       <c r="I17" s="33" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="J17">
         <v>643</v>
@@ -2492,11 +2512,11 @@
       <c r="H18" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I18" s="40" t="s">
+      <c r="I18" s="37" t="s">
+        <v>394</v>
+      </c>
+      <c r="J18" s="37" t="s">
         <v>395</v>
-      </c>
-      <c r="J18" s="40" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -2524,11 +2544,11 @@
       <c r="H19" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="I19" s="40" t="s">
+      <c r="I19" s="37" t="s">
+        <v>392</v>
+      </c>
+      <c r="J19" t="s">
         <v>393</v>
-      </c>
-      <c r="J19" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -2557,10 +2577,10 @@
         <v>28</v>
       </c>
       <c r="I20" s="33" t="s">
+        <v>390</v>
+      </c>
+      <c r="J20" s="33" t="s">
         <v>391</v>
-      </c>
-      <c r="J20" s="33" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -2589,10 +2609,10 @@
         <v>28</v>
       </c>
       <c r="I21" s="34" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="J21" s="34" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -2601,19 +2621,19 @@
         <v>234</v>
       </c>
       <c r="C22" s="16" t="s">
+        <v>383</v>
+      </c>
+      <c r="D22" s="16" t="s">
         <v>384</v>
-      </c>
-      <c r="D22" s="16" t="s">
-        <v>385</v>
       </c>
       <c r="E22" s="22"/>
       <c r="F22" s="16"/>
       <c r="G22" s="16"/>
       <c r="H22" s="18"/>
-      <c r="I22" s="39" t="s">
-        <v>386</v>
-      </c>
-      <c r="J22" s="39">
+      <c r="I22" s="36" t="s">
+        <v>385</v>
+      </c>
+      <c r="J22" s="36">
         <v>208</v>
       </c>
     </row>
@@ -2626,16 +2646,16 @@
         <v>202</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="E23" s="22"/>
       <c r="F23" s="16"/>
       <c r="G23" s="16"/>
       <c r="H23" s="18"/>
-      <c r="I23" s="39" t="s">
-        <v>388</v>
-      </c>
-      <c r="J23" s="39">
+      <c r="I23" s="36" t="s">
+        <v>387</v>
+      </c>
+      <c r="J23" s="36">
         <v>709</v>
       </c>
     </row>
@@ -2664,33 +2684,33 @@
       <c r="H24" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="I24" s="39" t="s">
+      <c r="I24" s="36" t="s">
+        <v>388</v>
+      </c>
+      <c r="J24" t="s">
         <v>389</v>
-      </c>
-      <c r="J24" t="s">
-        <v>390</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="19"/>
       <c r="B25" s="20" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C25" s="20" t="s">
+        <v>370</v>
+      </c>
+      <c r="D25" s="20" t="s">
         <v>371</v>
-      </c>
-      <c r="D25" s="20" t="s">
-        <v>372</v>
       </c>
       <c r="E25" s="22"/>
       <c r="F25" s="20"/>
       <c r="G25" s="20"/>
       <c r="H25" s="21"/>
       <c r="I25" t="s">
+        <v>372</v>
+      </c>
+      <c r="J25" t="s">
         <v>373</v>
-      </c>
-      <c r="J25" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -2699,39 +2719,39 @@
         <v>283</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E26" s="22"/>
       <c r="F26" s="20"/>
       <c r="G26" s="20"/>
       <c r="H26" s="21"/>
       <c r="I26" t="s">
+        <v>375</v>
+      </c>
+      <c r="J26" t="s">
         <v>376</v>
-      </c>
-      <c r="J26" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="19"/>
       <c r="B27" s="20" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C27" s="20" t="s">
+        <v>377</v>
+      </c>
+      <c r="D27" s="20" t="s">
         <v>378</v>
-      </c>
-      <c r="D27" s="20" t="s">
-        <v>379</v>
       </c>
       <c r="E27" s="22"/>
       <c r="F27" s="20"/>
       <c r="G27" s="20"/>
       <c r="H27" s="21"/>
       <c r="I27" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="J27">
         <v>20</v>
@@ -2742,13 +2762,13 @@
         <v>19</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="D28" s="16" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E28" s="22" t="s">
         <v>7</v>
@@ -2763,10 +2783,10 @@
         <v>28</v>
       </c>
       <c r="I28" s="34" t="s">
+        <v>381</v>
+      </c>
+      <c r="J28" s="34" t="s">
         <v>382</v>
-      </c>
-      <c r="J28" s="34" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -2774,7 +2794,7 @@
         <v>20</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C29" s="20" t="s">
         <v>118</v>
@@ -2795,10 +2815,10 @@
         <v>28</v>
       </c>
       <c r="I29" s="33" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J29" s="33" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -2856,7 +2876,7 @@
         <v>28</v>
       </c>
       <c r="I31" s="33" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -2885,7 +2905,7 @@
         <v>28</v>
       </c>
       <c r="I32" s="34" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -2914,10 +2934,10 @@
         <v>28</v>
       </c>
       <c r="I33" s="33" t="s">
+        <v>359</v>
+      </c>
+      <c r="J33" s="33" t="s">
         <v>360</v>
-      </c>
-      <c r="J33" s="33" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -2946,10 +2966,10 @@
         <v>28</v>
       </c>
       <c r="I34" s="34" t="s">
+        <v>357</v>
+      </c>
+      <c r="J34" s="34" t="s">
         <v>358</v>
-      </c>
-      <c r="J34" s="34" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -2978,7 +2998,7 @@
         <v>28</v>
       </c>
       <c r="I35" s="33" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="J35">
         <v>641</v>
@@ -3010,7 +3030,7 @@
         <v>28</v>
       </c>
       <c r="I36" s="34" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="J36">
         <v>671</v>
@@ -3042,10 +3062,10 @@
         <v>28</v>
       </c>
       <c r="I37" s="33" t="s">
+        <v>353</v>
+      </c>
+      <c r="J37" s="33" t="s">
         <v>354</v>
-      </c>
-      <c r="J37" s="33" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -3074,7 +3094,7 @@
         <v>28</v>
       </c>
       <c r="I38" s="34" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
@@ -3308,6 +3328,9 @@
       <c r="I46" s="34" t="s">
         <v>332</v>
       </c>
+      <c r="J46" s="34" t="s">
+        <v>413</v>
+      </c>
     </row>
     <row r="47" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="19">
@@ -3572,6 +3595,9 @@
       <c r="I55" s="31" t="s">
         <v>322</v>
       </c>
+      <c r="J55" t="s">
+        <v>414</v>
+      </c>
     </row>
     <row r="56" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="15">
@@ -3995,6 +4021,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J69" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>